<commit_message>
Jager Explica: vídeo real con persona, sin animación ni personaje
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013kFn69JUwjpJLGjYQm3cxD
</commit_message>
<xml_diff>
--- a/ESTUDIO/PEDIDOS_PIXELIDO/briefing_pixelido_canales.xlsx
+++ b/ESTUDIO/PEDIDOS_PIXELIDO/briefing_pixelido_canales.xlsx
@@ -878,7 +878,7 @@
       </c>
       <c r="C6" s="83" t="inlineStr">
         <is>
-          <t>Animación divertida en 3D cartoon, colores vivos y saturados, comparaciones absurdas ilustradas literalmente y ritmo rápido. Texto amarillo con contorno negro. Sellos recurrentes en pantalla: CIENCIA / HISTORIA (dato real) e IMAGINANDO (especulación). Personaje propio del canal como guía (diseño pendiente de definir; mientras tanto, un guía genérico de dibujos animados).</t>
+          <t>Vídeo real, no animación: imágenes y clips reales o de archivo, recreaciones realistas y gráficos sencillos, colores vivos y ritmo rápido. En algunos momentos aparece una persona como guía (sin animar). Las comparaciones absurdas se muestran de forma visual. Texto en pantalla amarillo con contorno negro. Sellos recurrentes: CIENCIA / HISTORIA (dato real) e IMAGINANDO (especulación). Sin personaje animado.</t>
         </is>
       </c>
       <c r="D6" s="83" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="G6" s="83" t="inlineStr">
         <is>
-          <t>Canal de divulgación con humor: escenarios hipotéticos («¿Y si…?») de ciencia e historia explicados con animación, separando lo real de lo imaginado. Vídeos largos de unos 20-25 minutos.</t>
+          <t>Canal de divulgación con humor: escenarios hipotéticos («¿Y si…?») de ciencia e historia contados con vídeo real y, en algunos momentos, una persona como guía, separando lo real de lo imaginado. Vídeos largos de unos 20-25 minutos.</t>
         </is>
       </c>
       <c r="H6" s="83" t="inlineStr">

</xml_diff>

<commit_message>
Jager Explica: vídeo normal sin persona ni personaje
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013kFn69JUwjpJLGjYQm3cxD
</commit_message>
<xml_diff>
--- a/ESTUDIO/PEDIDOS_PIXELIDO/briefing_pixelido_canales.xlsx
+++ b/ESTUDIO/PEDIDOS_PIXELIDO/briefing_pixelido_canales.xlsx
@@ -878,7 +878,7 @@
       </c>
       <c r="C6" s="83" t="inlineStr">
         <is>
-          <t>Vídeo real, no animación: imágenes y clips reales o de archivo, recreaciones realistas y gráficos sencillos, colores vivos y ritmo rápido. En algunos momentos aparece una persona como guía (sin animar). Las comparaciones absurdas se muestran de forma visual. Texto en pantalla amarillo con contorno negro. Sellos recurrentes: CIENCIA / HISTORIA (dato real) e IMAGINANDO (especulación). Sin personaje animado.</t>
+          <t>Vídeo normal, no animación: imágenes y clips reales o de archivo, recreaciones realistas y gráficos sencillos, colores vivos y ritmo rápido. Sin personaje ni presentador. Las comparaciones absurdas se muestran de forma visual. Texto en pantalla amarillo con contorno negro. Sellos recurrentes: CIENCIA / HISTORIA (dato real) e IMAGINANDO (especulación).</t>
         </is>
       </c>
       <c r="D6" s="83" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="G6" s="83" t="inlineStr">
         <is>
-          <t>Canal de divulgación con humor: escenarios hipotéticos («¿Y si…?») de ciencia e historia contados con vídeo real y, en algunos momentos, una persona como guía, separando lo real de lo imaginado. Vídeos largos de unos 20-25 minutos.</t>
+          <t>Canal de divulgación con humor: escenarios hipotéticos («¿Y si…?») de ciencia e historia contados con vídeo normal (imágenes reales y recreaciones), separando lo real de lo imaginado. Vídeos largos de unos 20-25 minutos.</t>
         </is>
       </c>
       <c r="H6" s="83" t="inlineStr">

</xml_diff>